<commit_message>
Drop answers and shared packages, plain UI wording, repo image names
Round 1 packages now always belong to a team and neither round stores
answers. image_url takes a file name from images/. Save status and
settings use plain Vietnamese with no technical terms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/gameshow-template.xlsx
+++ b/sheet-template/gameshow-template.xlsx
@@ -178,7 +178,7 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Link ảnh đội (tùy chọn). Trống thì dùng chữ viết tắt tên đội.</t>
+        <t>Tên file ảnh đội trong thư mục images/ (vd: doi-01.jpg). Trống thì dùng chữ viết tắt tên đội.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
@@ -198,12 +198,12 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Tên gói câu hỏi. Mỗi gói = 1 câu hỏi (1 dòng).</t>
+        <t>Tên gói câu hỏi. Mỗi gói = 1 câu hỏi (1 dòng). Bắt buộc.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Mã đội sở hữu gói (tùy chọn). Trống = gói chung, đội nào chọn trước thì khóa với đội khác.</t>
+        <t>Mã đội sở hữu gói (vd: doi-01). Bắt buộc.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -213,20 +213,15 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Đáp án (tùy chọn, không hiện trên màn hình).</t>
+        <t>Tên file ảnh minh họa trong thư mục images/ (tùy chọn).</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Link ảnh minh họa (tùy chọn).</t>
+        <t>Thời gian trả lời (giây). Trống = dùng round1_time_seconds trong tab config.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Thời gian trả lời (giây). Trống = dùng round1_time_seconds trong tab config.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Điểm của câu hỏi. Trống = dùng giá trị mặc định trong config.</t>
       </text>
@@ -253,20 +248,15 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Đáp án (tùy chọn).</t>
+        <t>Tên file ảnh minh họa trong thư mục images/ (tùy chọn).</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Link ảnh minh họa (tùy chọn).</t>
+        <t>Thời gian trả lời (giây). Trống = dùng round3_time_seconds trong config.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Thời gian trả lời (giây). Trống = dùng round3_time_seconds trong config.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Điểm của ô. Trống = dùng giá trị mặc định trong config.</t>
       </text>
@@ -937,16 +927,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -967,20 +956,15 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>answer</t>
+          <t>image_url</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>image_url</t>
+          <t>time_seconds</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>time_seconds</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>points</t>
         </is>
@@ -1002,16 +986,11 @@
           <t>Kinh đô của nhà nước Văn Lang được đặt tại vùng đất thuộc tỉnh nào của Việt Nam hiện nay?</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Phú Thọ</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr"/>
+      <c r="E2" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F2" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G2" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1031,16 +1010,11 @@
           <t>Nguyên tố hóa học nào chiếm tỷ lệ thể tích lớn nhất trong khí quyển Trái Đất?</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Nitơ (khoảng 78%)</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr"/>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F3" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G3" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1060,16 +1034,11 @@
           <t>Tác phẩm "Truyện Kiều" của đại thi hào Nguyễn Du được viết theo thể thơ nào?</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Thể thơ lục bát</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G4" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1089,16 +1058,11 @@
           <t>Ánh sáng từ Mặt Trời mất khoảng bao nhiêu phút để truyền tới Trái Đất?</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Khoảng 8 phút 20 giây</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F5" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G5" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1118,16 +1082,11 @@
           <t>Sông Mê Kông chảy vào lãnh thổ Việt Nam qua hai nhánh chính là sông Tiền và sông gì?</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Sông Hậu</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G6" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1147,16 +1106,11 @@
           <t>Từ viết tắt "CPU" trong máy tính có nghĩa tiếng Việt là gì?</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Bộ xử lý trung tâm</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F7" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G7" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1176,16 +1130,11 @@
           <t>Quần thể di tích Cố đô Huế được UNESCO công nhận là Di sản Văn hóa Thế giới vào năm nào?</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Năm 1993</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G8" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1205,16 +1154,11 @@
           <t>Quá trình cây xanh tổng hợp chất hữu cơ nhờ năng lượng ánh sáng gọi là gì?</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Quang hợp</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F9" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G9" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1234,16 +1178,11 @@
           <t>Vị vua nào đã ban "Chiếu dời đô" đưa kinh đô từ Hoa Lư về Đại La (Thăng Long) năm 1010?</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Lý Thái Tổ (Lý Công Uẩn)</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F10" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G10" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1263,16 +1202,11 @@
           <t>Đại dương nào có diện tích và độ sâu lớn nhất thế giới?</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Thái Bình Dương</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F11" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G11" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1292,16 +1226,11 @@
           <t>Lễ hội Đền Hùng tưởng nhớ các Vua Hùng diễn ra vào ngày nào âm lịch hằng năm?</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Mùng 10 tháng 3 âm lịch</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F12" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G12" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1321,366 +1250,299 @@
           <t>Trong bảng tuần hoàn hóa học, nguyên tố Vàng có ký hiệu là gì?</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Au</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F13" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G13" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 01</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr"/>
+          <t>Gói A</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>doi-07</t>
+        </is>
+      </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Tác giả của bản "Tuyên ngôn Độc lập" khai sinh nước Việt Nam Dân chủ Cộng hòa ngày 2/9/1945 là ai?</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Chủ tịch Hồ Chí Minh</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F14" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G14" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 02</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr"/>
+          <t>Gói B</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>doi-07</t>
+        </is>
+      </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Chiến dịch Hồ Chí Minh lịch sử toàn thắng vào ngày tháng năm nào?</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>30/04/1975</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F15" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G15" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 03</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr"/>
+          <t>Gói A</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>doi-08</t>
+        </is>
+      </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Trường đại học đầu tiên của Việt Nam tại kinh thành Thăng Long có tên là gì?</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Quốc Tử Giám</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F16" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G16" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 04</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr"/>
+          <t>Gói B</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>doi-08</t>
+        </is>
+      </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Trên sông Bạch Đằng năm 938, vị anh hùng nào đã đánh tan quân Nam Hán?</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Ngô Quyền</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F17" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G17" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 05</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr"/>
+          <t>Gói A</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>doi-09</t>
+        </is>
+      </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Ai là vị trạng nguyên trẻ tuổi nhất trong lịch sử khoa bảng phong kiến Việt Nam?</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Nguyễn Hiền</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F18" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G18" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 06</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
+          <t>Gói B</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>doi-09</t>
+        </is>
+      </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Bài hát "Tiến quân ca" - Quốc ca Việt Nam do nhạc sĩ nào sáng tác?</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Văn Cao</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F19" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G19" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 07</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr"/>
+          <t>Gói A</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>doi-10</t>
+        </is>
+      </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Đảo lớn nhất của Việt Nam tính theo diện tích là đảo nào?</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Đảo Phú Quốc</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F20" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G20" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 08</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr"/>
+          <t>Gói B</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>doi-10</t>
+        </is>
+      </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Nhà Trần đã ba lần đánh thắng quân xâm lược Nguyên - Mông vào thế kỷ thứ mấy?</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Thế kỷ XIII</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr"/>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F21" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G21" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 09</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr"/>
+          <t>Gói A</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>doi-11</t>
+        </is>
+      </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Chợ nổi Cái Răng là nét văn hóa đặc sắc của thành phố trực thuộc trung ương nào?</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Thành phố Cần Thơ</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F22" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G22" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 10</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr"/>
+          <t>Gói B</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>doi-11</t>
+        </is>
+      </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Cao nguyên đá Đồng Văn nằm ở tỉnh nào của nước ta?</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Tỉnh Hà Giang</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F23" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G23" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 11</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr"/>
+          <t>Gói A</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>doi-12</t>
+        </is>
+      </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Ai là tác giả của "Bình Ngô đại cáo" - bản tuyên ngôn độc lập thứ hai của dân tộc?</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Nguyễn Trãi</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F24" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G24" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Gói Chung 12</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr"/>
+          <t>Gói B</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>doi-12</t>
+        </is>
+      </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Bài thơ thần "Nam quốc sơn hà" tương truyền vang lên bên dòng sông nào?</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Sông Như Nguyệt</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="n">
+        <v>15</v>
+      </c>
       <c r="F25" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Gói Chung 13</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Hồ nước ngọt tự nhiên lớn nhất miền núi phía Bắc Việt Nam là hồ nào?</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Hồ Ba Bể</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Gói Chung 14</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Đèo Hải Vân nằm giữa ranh giới tỉnh Thừa Thiên Huế và thành phố nào?</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Thành phố Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G27" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1696,15 +1558,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="51" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1720,20 +1581,15 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>answer</t>
+          <t>image_url</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>image_url</t>
+          <t>time_seconds</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>time_seconds</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>points</t>
         </is>
@@ -1748,16 +1604,11 @@
           <t>Nhà nước đầu tiên trong lịch sử dân tộc Việt Nam có tên gọi là gì?</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Nhà nước Văn Lang</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr"/>
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E2" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F2" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1770,16 +1621,11 @@
           <t>Sông nào dài nhất trên thế giới chảy qua khu vực Đông Bắc châu Phi?</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Sông Nin (Nile)</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr"/>
+      <c r="C3" s="4" t="inlineStr"/>
+      <c r="D3" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E3" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F3" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1792,16 +1638,11 @@
           <t>Nguyên tố hóa học nào có số hiệu nguyên tử bằng 1 trong bảng tuần hoàn?</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Hiđrô (H)</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F4" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1814,16 +1655,11 @@
           <t>Tác phẩm "Nhật ký trong tù" của Chủ tịch Hồ Chí Minh được viết bằng chữ gì?</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Chữ Hán</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E5" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F5" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1836,16 +1672,11 @@
           <t>Thành phố nào là thủ đô của nước Cộng hòa Nhân dân Trung Hoa?</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Bắc Kinh</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E6" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F6" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1858,16 +1689,11 @@
           <t>Trong hình học phẳng, đường thẳng đi qua tâm và nối hai điểm trên đường tròn gọi là gì?</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Đường kính</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E7" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F7" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1880,16 +1706,11 @@
           <t>Vịnh biển nào của Việt Nam từng hai lần được UNESCO công nhận là Di sản Thiên nhiên Thế giới về giá trị thẩm mỹ và địa chất?</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Vịnh Hạ Long</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E8" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F8" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1902,16 +1723,11 @@
           <t>Ai là người chỉ huy quân dân nhà Trần lập chiến công trên sông Bạch Đằng năm 1288?</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Trần Hưng Đạo (Hưng Đạo Đại Vương Trần Quốc Tuấn)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E9" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F9" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1924,16 +1740,11 @@
           <t>Hành tinh nào trong Hệ Mặt Trời nổi tiếng với hệ thống vành đai băng và bụi rộng lớn dễ quan sát nhất?</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Sao Thổ (Thổ tinh)</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E10" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1946,16 +1757,11 @@
           <t>Cơ quan hô hấp chính của loài cá sống dưới nước là bộ phận nào?</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Mang</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E11" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F11" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1968,16 +1774,11 @@
           <t>Tỉnh nào của Việt Nam có diện tích tự nhiên lớn nhất cả nước?</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Tỉnh Nghệ An</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E12" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F12" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1990,16 +1791,11 @@
           <t>Bản giao hưởng "Định mệnh" (Số 5) là kiệt tác của nhà soạn nhạc người Đức nào?</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Ludwig van Beethoven</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E13" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F13" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2012,16 +1808,11 @@
           <t>Đơn vị đo tần số dao động trong hệ đo lường quốc tế SI là gì?</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Héc (Hz - Hertz)</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E14" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F14" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2034,16 +1825,11 @@
           <t>Chiến dịch Điện Biên Phủ năm 1954 kéo dài trong bao nhiêu ngày đêm?</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>56 ngày đêm</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E15" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F15" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2056,16 +1842,11 @@
           <t>Quốc gia nào có diện tích lãnh thổ lớn nhất thế giới?</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Liên bang Nga</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E16" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F16" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2078,16 +1859,11 @@
           <t>Tác giả của truyện ngắn "Vợ nhặt" trong văn học Việt Nam hiện đại là ai?</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Kim Lân</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E17" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F17" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2100,16 +1876,11 @@
           <t>Kim loại nào nhẹ nhất (có khối lượng riêng nhỏ nhất) trong tất cả các kim loại ở điều kiện chuẩn?</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Liti (Li)</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E18" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F18" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2122,16 +1893,11 @@
           <t>Đường xích đạo chia quả địa cầu thành hai phần bằng nhau gọi là gì?</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Bán cầu Bắc và Bán cầu Nam</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E19" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F19" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2144,16 +1910,11 @@
           <t>Kinh thành Huế được xây dựng bắt đầu từ triều vua nào của nhà Nguyễn?</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Vua Gia Long</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E20" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F20" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2166,16 +1927,11 @@
           <t>Trong công nghệ thông tin, thuật ngữ "RAM" là viết tắt của cụm từ tiếng Anh nào?</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Random Access Memory (Bộ nhớ truy cập ngẫu nhiên)</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E21" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F21" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2188,16 +1944,11 @@
           <t>Loài cây nào thường được xem là biểu tượng cho phẩm chất thanh cao, được đề cử là Quốc hoa Việt Nam?</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Hoa sen</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F22" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2210,16 +1961,11 @@
           <t>Ai là nhà bác học vĩ đại đã phát hiện ra định luật vạn vật hấp dẫn?</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Isaac Newton</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E23" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F23" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2232,16 +1978,11 @@
           <t>Thành cổ Quảng Trị gắn liền với cuộc chiến đấu 81 ngày đêm mùa hè đỏ lửa vào năm nào?</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Năm 1972</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E24" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F24" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2254,16 +1995,11 @@
           <t>Hồ nước ngọt sâu nhất trên thế giới nằm ở vùng Siberia (Nga) có tên là gì?</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Hồ Baikal</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E25" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F25" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2276,16 +2012,11 @@
           <t>Vitamin nào đóng vai trò quan trọng giúp tăng cường thị lực và phòng ngừa bệnh quáng gà?</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Vitamin A</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E26" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F26" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2298,16 +2029,11 @@
           <t>Tác phẩm "Số đỏ" với nhân vật Xuân Tóc Đỏ là tiểu thuyết trào phúng của nhà văn nào?</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Vũ Trọng Phụng</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E27" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F27" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2320,16 +2046,11 @@
           <t>Dãy núi Himalaya nằm ở châu lục nào?</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Châu Á</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E28" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F28" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2342,16 +2063,11 @@
           <t>Trong vật lý, đại lượng đặc trưng cho sự nhanh hay chậm của chuyển động gọi là gì?</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Vận tốc (hoặc tốc độ)</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr"/>
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E29" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F29" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2364,16 +2080,11 @@
           <t>Ai là nữ tướng đầu tiên của Quân đội Nhân dân Việt Nam?</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Nguyễn Thị Định</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E30" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F30" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2386,16 +2097,11 @@
           <t>Quần đảo Hoàng Sa trực thuộc đơn vị hành chính cấp tỉnh/thành phố nào của Việt Nam?</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Thành phố Đà Nẵng</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr"/>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E31" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F31" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2408,16 +2114,11 @@
           <t>Chất khí nào gây ra hiệu ứng nhà kính mạnh mẽ nhất do hoạt động đốt nhiên liệu hóa thạch của con người?</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Khí Cacbon đioxit (CO2)</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr"/>
+      <c r="C32" s="4" t="inlineStr"/>
+      <c r="D32" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E32" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F32" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2430,16 +2131,11 @@
           <t>Bài thơ "Đất Nước" (trích trường ca Mặt đường khát vọng) là sáng tác của nhà thơ nào?</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Nguyễn Khoa Điềm</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E33" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F33" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2452,16 +2148,11 @@
           <t>Eo biển nào ngăn cách đảo Anh với lục địa châu Âu?</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Eo biển Manche (English Channel)</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E34" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F34" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2474,16 +2165,11 @@
           <t>Một byte trong tin học tương đương với bao nhiêu bit?</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>8 bit</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E35" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F35" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2496,16 +2182,11 @@
           <t>Phong trào Cần Vương cuối thế kỷ XIX được phát động bởi chiếu Cần Vương nhân danh vị vua nào?</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Vua Hàm Nghi</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E36" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F36" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2518,16 +2199,11 @@
           <t>Nhóm máu nào được gọi là nhóm máu "chuyên cho" (hồng cầu lắng) trong truyền máu cổ điển?</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Nhóm máu O (O Rh-)</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E37" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F37" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2540,16 +2216,11 @@
           <t>Sông Hồng chảy vào địa phận Việt Nam đầu tiên tại tỉnh nào?</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Tỉnh Lào Cai</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E38" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F38" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2562,16 +2233,11 @@
           <t>Tác giả của thuyết tương đối rộng và thuyết tương đối hẹp trong vật lý hiện đại là ai?</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Albert Einstein</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr"/>
+      <c r="D39" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E39" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F39" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2584,16 +2250,11 @@
           <t>Di sản Văn hóa Thế giới Phố cổ Hội An nằm bên bờ con sông nào?</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Sông Thu Bồn (nhánh sông Hoài)</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E40" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F40" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2606,16 +2267,11 @@
           <t>Hợp kim đồng thau là sự kết hợp chủ yếu giữa kim loại đồng (Cu) và kim loại nào?</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Kẽm (Zn)</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="n">
+        <v>30</v>
+      </c>
       <c r="E41" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F41" s="4" t="n">
         <v>40</v>
       </c>
     </row>
@@ -2628,16 +2284,11 @@
           <t>Hiệp định Genève về chấm dứt chiến tranh, lập lại hòa bình ở Đông Dương được ký kết vào năm nào?</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Năm 1954</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E42" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F42" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2650,16 +2301,11 @@
           <t>Châu lục nào nằm hoàn toàn ở bán cầu Nam và được bao phủ bởi băng tuyết quanh năm?</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Châu Nam Cực</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr"/>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E43" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F43" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2672,16 +2318,11 @@
           <t>Nhà bác học Marie Curie đã tìm ra hai nguyên tố phóng xạ nào?</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Poloni (Po) và Rađi (Ra)</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="n">
+        <v>30</v>
+      </c>
       <c r="E44" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F44" s="4" t="n">
         <v>40</v>
       </c>
     </row>
@@ -2694,16 +2335,11 @@
           <t>Trong văn học dân gian Việt Nam, vị thần nào trong "Tứ bất tử" gắn với truyền thuyết chống lũ lụt sông Hồng?</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Sơn Tinh (Tản Viên Sơn Thánh)</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E45" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F45" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2716,16 +2352,11 @@
           <t>Ký hiệu hóa học của nguyên tố Sắt trong bảng tuần hoàn là gì?</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Fe</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E46" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F46" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2738,16 +2369,11 @@
           <t>Hiệp hội các quốc gia Đông Nam Á (ASEAN) được thành lập vào năm nào?</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Năm 1967</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="E47" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="F47" s="4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2760,16 +2386,11 @@
           <t>Đỉnh núi cao nhất trên Trái Đất thuộc dãy Himalaya có tên là gì?</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Đỉnh Everest (Chomolungma)</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E48" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F48" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2782,16 +2403,11 @@
           <t>Ai là người Việt Nam đầu tiên bay vào vũ trụ trên tàu Liên hợp 37 năm 1980?</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>Phạm Tuân</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr"/>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E49" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F49" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2804,16 +2420,11 @@
           <t>Trong toán học, hằng số Pi (tỷ số giữa chu vi và đường kính đường tròn) có giá trị xấp xỉ hai chữ số thập phân là bao nhiêu?</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>3,14</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E50" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F50" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2826,16 +2437,11 @@
           <t>Bến Nhà Rồng - nơi người thanh niên Nguyễn Tất Thành ra đi tìm đường cứu nước năm 1911 - nằm tại thành phố nào hiện nay?</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>Thành phố Hồ Chí Minh</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr"/>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="E51" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F51" s="4" t="n">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add per-person accounts, short home page, touch judge sheet, sync fixes
Logins come from an accounts sheet tab (defaults mc, gk1.., doi01..)
and route each person to their portal as that judge or team; each role
keeps its own login slot. The home page is three icon tiles. The judge
screen uses large steppers and quick-pick scores with a team overview.

Fixes: collapsed sidebar shows only the status dot; host pages were
blank after login; a sheet load error no longer logs devices out; a
stale data cache is ignored; judge and team screens replace their live
copy on each update, so a reset or a cleared stage reaches them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/gameshow-template.xlsx
+++ b/sheet-template/gameshow-template.xlsx
@@ -13,7 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="round2" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="round3" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="judges" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="accounts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -354,12 +355,47 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
+        <t>Tên đăng nhập (không phân biệt hoa thường). Bắt buộc, duy nhất.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Mật khẩu đăng nhập (văn bản thuần). Bắt buộc.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Vai trò: host (dẫn chương trình), judge (giám khảo), hoặc team (đội thi). Bắt buộc.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Mã giám khảo (từ tab judges) hoặc mã đội (từ tab teams). Để trống với host.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Tên hiển thị người dùng (tùy chọn).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Mẫu</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
         <t>Tên cài đặt (key). Không đổi tên cột key.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Giá trị cài đặt (tên hội thi, thời gian, điểm tối đa, mật khẩu sha256...).</t>
+        <t>Giá trị cài đặt (tên hội thi, thời gian, điểm tối đa, màu giao diện...).</t>
       </text>
     </comment>
   </commentList>
@@ -681,7 +717,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2. Giữ nguyên TÊN CÁC TAB (teams, round1, round2, round3, judges, config) và TÊN CỘT ở dòng 1 (ô màu cam).</t>
+          <t>2. Giữ nguyên TÊN CÁC TAB (teams, round1, round2, round3, judges, accounts, config) và TÊN CỘT ở dòng 1 (ô màu cam).</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2990,484 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>password</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>ref_id</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>mc</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Dẫn chương trình</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>gk1</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>judge</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>gk-01</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Ban Giám khảo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>gk2</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>judge</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>gk-02</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Ban Giám khảo 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>gk3</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>judge</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>gk-03</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Ban Giám khảo 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>doi01</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>doi-01</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Đội Sao Vàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>doi02</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>doi-02</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Đội Hồng Hà</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>doi03</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>doi-03</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Đội Cửu Long</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>doi04</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>doi-04</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Đội Trường Sơn</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>doi05</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>doi-05</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Đội Đông Đô</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>doi06</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>doi-06</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Đội Lam Sơn</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>doi07</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>doi-07</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Đội Bạch Đằng</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>doi08</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>doi-08</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Đội Thăng Long</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>doi09</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>doi-09</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Đội Phù Đổng</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>doi10</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>doi-10</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Đội Vạn Xuân</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>doi11</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>doi-11</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Đội Đại Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>doi12</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>122345678910</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>doi-12</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Đội Âu Lạc</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3240,118 +3753,94 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>password_host_sha256</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr"/>
+          <t>theme_mode</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>password_judge_sha256</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr"/>
+          <t>bg_color</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>#F5F4ED</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>password_team_sha256</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr"/>
+          <t>surface_color</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>#FAF9F5</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>theme_mode</t>
+          <t>text_color</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>#141413</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>bg_color</t>
+          <t>muted_color</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>#F5F4ED</t>
+          <t>#6B6960</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>surface_color</t>
+          <t>accent_color</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>#FAF9F5</t>
+          <t>#D97757</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>text_color</t>
+          <t>accent_dark_color</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>#141413</t>
+          <t>#C6613F</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>muted_color</t>
+          <t>border_color</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>#6B6960</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>accent_color</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>#D97757</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>accent_dark_color</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>#C6613F</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>border_color</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>#E3E0D3</t>
         </is>

</xml_diff>